<commit_message>
commit: Proyecto Impresiones Express listo
</commit_message>
<xml_diff>
--- a/dataset_impresiones_100_estricto.xlsx
+++ b/dataset_impresiones_100_estricto.xlsx
@@ -418,16 +418,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kristel 45</v>
+        <v>Smart Fit 42</v>
       </c>
       <c r="B2" t="str">
-        <v>gran_formato</v>
+        <v>offset</v>
       </c>
       <c r="C2" t="str">
-        <v>A1</v>
+        <v>A2</v>
       </c>
       <c r="D2">
-        <v>1602</v>
+        <v>1200</v>
       </c>
       <c r="E2" t="str">
         <v>papel_couche</v>
@@ -435,33 +435,33 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Jesus 3</v>
+        <v>Alejandro 79</v>
       </c>
       <c r="B3" t="str">
-        <v>offset</v>
+        <v>digital</v>
       </c>
       <c r="C3" t="str">
         <v>personalizado</v>
       </c>
       <c r="D3">
-        <v>113</v>
+        <v>3560</v>
       </c>
       <c r="E3" t="str">
-        <v>cartulina</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Kristel 79</v>
+        <v>Alejandro 1</v>
       </c>
       <c r="B4" t="str">
         <v>gran_formato</v>
       </c>
       <c r="C4" t="str">
-        <v>A2</v>
+        <v>A1</v>
       </c>
       <c r="D4">
-        <v>1566</v>
+        <v>3377</v>
       </c>
       <c r="E4" t="str">
         <v>vinilo</v>
@@ -469,50 +469,50 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Jesus 7</v>
+        <v>Smart Fit 12</v>
       </c>
       <c r="B5" t="str">
         <v>gran_formato</v>
       </c>
       <c r="C5" t="str">
-        <v>A4</v>
+        <v>personalizado</v>
       </c>
       <c r="D5">
-        <v>3521</v>
+        <v>3674</v>
       </c>
       <c r="E5" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Clínica Rene 14</v>
+        <v>Smart Fit 17</v>
       </c>
       <c r="B6" t="str">
-        <v>serigrafia</v>
+        <v>gran_formato</v>
       </c>
       <c r="C6" t="str">
-        <v>personalizado</v>
+        <v>A1</v>
       </c>
       <c r="D6">
-        <v>699</v>
+        <v>1565</v>
       </c>
       <c r="E6" t="str">
-        <v>papel_bond</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Alejandro 34</v>
+        <v>Noemi 92</v>
       </c>
       <c r="B7" t="str">
-        <v>digital</v>
+        <v>serigrafia</v>
       </c>
       <c r="C7" t="str">
-        <v>A0</v>
+        <v>A3</v>
       </c>
       <c r="D7">
-        <v>3627</v>
+        <v>3413</v>
       </c>
       <c r="E7" t="str">
         <v>papel_bond</v>
@@ -520,50 +520,50 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Clínica Rene 66</v>
+        <v>Alejandro 1</v>
       </c>
       <c r="B8" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C8" t="str">
-        <v>A2</v>
+        <v>A3</v>
       </c>
       <c r="D8">
-        <v>40</v>
+        <v>486</v>
       </c>
       <c r="E8" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Clínica Rene 8</v>
+        <v>Smart Fit 63</v>
       </c>
       <c r="B9" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C9" t="str">
-        <v>A3</v>
+        <v>A0</v>
       </c>
       <c r="D9">
-        <v>4245</v>
+        <v>751</v>
       </c>
       <c r="E9" t="str">
-        <v>papel_bond</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Smart Fit 45</v>
+        <v>Alejandro 99</v>
       </c>
       <c r="B10" t="str">
-        <v>digital</v>
+        <v>serigrafia</v>
       </c>
       <c r="C10" t="str">
         <v>A1</v>
       </c>
       <c r="D10">
-        <v>452</v>
+        <v>2572</v>
       </c>
       <c r="E10" t="str">
         <v>papel_bond</v>
@@ -571,16 +571,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>UTP 47</v>
+        <v>ModoDía 94</v>
       </c>
       <c r="B11" t="str">
-        <v>gran_formato</v>
+        <v>offset</v>
       </c>
       <c r="C11" t="str">
-        <v>A3</v>
+        <v>A0</v>
       </c>
       <c r="D11">
-        <v>2908</v>
+        <v>3919</v>
       </c>
       <c r="E11" t="str">
         <v>papel_couche</v>
@@ -588,135 +588,135 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Clínica Rene 23</v>
+        <v>Smart Fit 93</v>
       </c>
       <c r="B12" t="str">
-        <v>offset</v>
+        <v>serigrafia</v>
       </c>
       <c r="C12" t="str">
         <v>A3</v>
       </c>
       <c r="D12">
-        <v>83</v>
+        <v>3707</v>
       </c>
       <c r="E12" t="str">
-        <v>papel_couche</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Alejandro 84</v>
+        <v>Tottus 35</v>
       </c>
       <c r="B13" t="str">
-        <v>digital</v>
+        <v>serigrafia</v>
       </c>
       <c r="C13" t="str">
         <v>A2</v>
       </c>
       <c r="D13">
-        <v>1635</v>
+        <v>1307</v>
       </c>
       <c r="E13" t="str">
-        <v>cartulina</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Smart Fit 20</v>
+        <v>Tottus 62</v>
       </c>
       <c r="B14" t="str">
-        <v>serigrafia</v>
+        <v>digital</v>
       </c>
       <c r="C14" t="str">
-        <v>A3</v>
+        <v>A0</v>
       </c>
       <c r="D14">
-        <v>4070</v>
+        <v>4737</v>
       </c>
       <c r="E14" t="str">
-        <v>cartulina</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Smart Fit 14</v>
+        <v>UTP 79</v>
       </c>
       <c r="B15" t="str">
-        <v>serigrafia</v>
+        <v>offset</v>
       </c>
       <c r="C15" t="str">
-        <v>personalizado</v>
+        <v>A2</v>
       </c>
       <c r="D15">
-        <v>4404</v>
+        <v>2068</v>
       </c>
       <c r="E15" t="str">
-        <v>cartulina</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Kristel 89</v>
+        <v>Clínica Rene 76</v>
       </c>
       <c r="B16" t="str">
         <v>serigrafia</v>
       </c>
       <c r="C16" t="str">
-        <v>A2</v>
+        <v>A1</v>
       </c>
       <c r="D16">
-        <v>2451</v>
+        <v>1058</v>
       </c>
       <c r="E16" t="str">
-        <v>cartulina</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Noemi 21</v>
+        <v>UTP 22</v>
       </c>
       <c r="B17" t="str">
         <v>serigrafia</v>
       </c>
       <c r="C17" t="str">
-        <v>A3</v>
+        <v>A1</v>
       </c>
       <c r="D17">
-        <v>473</v>
+        <v>3475</v>
       </c>
       <c r="E17" t="str">
-        <v>lona</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Smart Fit 21</v>
+        <v>Sofia 11</v>
       </c>
       <c r="B18" t="str">
-        <v>offset</v>
+        <v>gran_formato</v>
       </c>
       <c r="C18" t="str">
-        <v>A1</v>
+        <v>personalizado</v>
       </c>
       <c r="D18">
-        <v>2177</v>
+        <v>1043</v>
       </c>
       <c r="E18" t="str">
-        <v>vinilo</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Alejandro 49</v>
+        <v>Joselin 53</v>
       </c>
       <c r="B19" t="str">
-        <v>gran_formato</v>
+        <v>offset</v>
       </c>
       <c r="C19" t="str">
-        <v>personalizado</v>
+        <v>A4</v>
       </c>
       <c r="D19">
-        <v>4520</v>
+        <v>3493</v>
       </c>
       <c r="E19" t="str">
         <v>cartulina</v>
@@ -724,84 +724,84 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ModoDía 40</v>
+        <v>Tottus 51</v>
       </c>
       <c r="B20" t="str">
         <v>offset</v>
       </c>
       <c r="C20" t="str">
-        <v>A4</v>
+        <v>A3</v>
       </c>
       <c r="D20">
-        <v>1404</v>
+        <v>1880</v>
       </c>
       <c r="E20" t="str">
-        <v>papel_couche</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Alejandro 77</v>
+        <v>Noemi 1</v>
       </c>
       <c r="B21" t="str">
-        <v>serigrafia</v>
+        <v>offset</v>
       </c>
       <c r="C21" t="str">
-        <v>A4</v>
+        <v>personalizado</v>
       </c>
       <c r="D21">
-        <v>4489</v>
+        <v>1411</v>
       </c>
       <c r="E21" t="str">
-        <v>vinilo</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Noemi 61</v>
+        <v>Tottus 22</v>
       </c>
       <c r="B22" t="str">
-        <v>serigrafia</v>
+        <v>digital</v>
       </c>
       <c r="C22" t="str">
-        <v>A2</v>
+        <v>A3</v>
       </c>
       <c r="D22">
-        <v>3035</v>
+        <v>2618</v>
       </c>
       <c r="E22" t="str">
-        <v>vinilo</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Smart Fit 25</v>
+        <v>Tottus 87</v>
       </c>
       <c r="B23" t="str">
-        <v>gran_formato</v>
+        <v>digital</v>
       </c>
       <c r="C23" t="str">
-        <v>A3</v>
+        <v>A0</v>
       </c>
       <c r="D23">
-        <v>601</v>
+        <v>4026</v>
       </c>
       <c r="E23" t="str">
-        <v>lona</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Noemi 19</v>
+        <v>Tottus 55</v>
       </c>
       <c r="B24" t="str">
-        <v>digital</v>
+        <v>gran_formato</v>
       </c>
       <c r="C24" t="str">
-        <v>personalizado</v>
+        <v>A1</v>
       </c>
       <c r="D24">
-        <v>3436</v>
+        <v>2681</v>
       </c>
       <c r="E24" t="str">
         <v>papel_bond</v>
@@ -809,441 +809,441 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Clínica Rene 49</v>
+        <v>Jesus 43</v>
       </c>
       <c r="B25" t="str">
         <v>serigrafia</v>
       </c>
       <c r="C25" t="str">
-        <v>A4</v>
+        <v>A0</v>
       </c>
       <c r="D25">
-        <v>3807</v>
+        <v>4310</v>
       </c>
       <c r="E25" t="str">
-        <v>cartulina</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Kristel 37</v>
+        <v>Kristel 8</v>
       </c>
       <c r="B26" t="str">
         <v>offset</v>
       </c>
       <c r="C26" t="str">
-        <v>A0</v>
+        <v>A2</v>
       </c>
       <c r="D26">
-        <v>4778</v>
+        <v>2531</v>
       </c>
       <c r="E26" t="str">
-        <v>papel_couche</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Noemi 91</v>
+        <v>Joselin 96</v>
       </c>
       <c r="B27" t="str">
-        <v>gran_formato</v>
+        <v>serigrafia</v>
       </c>
       <c r="C27" t="str">
         <v>personalizado</v>
       </c>
       <c r="D27">
-        <v>3694</v>
+        <v>4159</v>
       </c>
       <c r="E27" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>UTP 45</v>
+        <v>Smart Fit 59</v>
       </c>
       <c r="B28" t="str">
-        <v>digital</v>
+        <v>serigrafia</v>
       </c>
       <c r="C28" t="str">
-        <v>A4</v>
+        <v>personalizado</v>
       </c>
       <c r="D28">
-        <v>681</v>
+        <v>4020</v>
       </c>
       <c r="E28" t="str">
-        <v>lona</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Tottus 22</v>
+        <v>Alejandro 24</v>
       </c>
       <c r="B29" t="str">
-        <v>serigrafia</v>
+        <v>offset</v>
       </c>
       <c r="C29" t="str">
-        <v>A0</v>
+        <v>A3</v>
       </c>
       <c r="D29">
-        <v>1064</v>
+        <v>4944</v>
       </c>
       <c r="E29" t="str">
-        <v>vinilo</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>UTP 27</v>
+        <v>Clínica Rene 47</v>
       </c>
       <c r="B30" t="str">
-        <v>serigrafia</v>
+        <v>offset</v>
       </c>
       <c r="C30" t="str">
-        <v>A4</v>
+        <v>A1</v>
       </c>
       <c r="D30">
-        <v>893</v>
+        <v>4429</v>
       </c>
       <c r="E30" t="str">
-        <v>cartulina</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Clínica Rene 27</v>
+        <v>Tottus 70</v>
       </c>
       <c r="B31" t="str">
         <v>digital</v>
       </c>
       <c r="C31" t="str">
-        <v>A0</v>
+        <v>A1</v>
       </c>
       <c r="D31">
-        <v>2861</v>
+        <v>1715</v>
       </c>
       <c r="E31" t="str">
-        <v>papel_couche</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Alejandro 13</v>
+        <v>UTP 27</v>
       </c>
       <c r="B32" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C32" t="str">
-        <v>A3</v>
+        <v>A2</v>
       </c>
       <c r="D32">
-        <v>2483</v>
+        <v>1194</v>
       </c>
       <c r="E32" t="str">
-        <v>lona</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Smart Fit 40</v>
+        <v>Kristel 19</v>
       </c>
       <c r="B33" t="str">
-        <v>digital</v>
+        <v>gran_formato</v>
       </c>
       <c r="C33" t="str">
-        <v>A3</v>
+        <v>A0</v>
       </c>
       <c r="D33">
-        <v>1853</v>
+        <v>3604</v>
       </c>
       <c r="E33" t="str">
-        <v>vinilo</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Kristel 38</v>
+        <v>Alejandro 56</v>
       </c>
       <c r="B34" t="str">
-        <v>offset</v>
+        <v>serigrafia</v>
       </c>
       <c r="C34" t="str">
-        <v>A4</v>
+        <v>A3</v>
       </c>
       <c r="D34">
-        <v>3810</v>
+        <v>2926</v>
       </c>
       <c r="E34" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Kristel 7</v>
+        <v>Joselin 17</v>
       </c>
       <c r="B35" t="str">
-        <v>offset</v>
+        <v>serigrafia</v>
       </c>
       <c r="C35" t="str">
-        <v>A2</v>
+        <v>personalizado</v>
       </c>
       <c r="D35">
-        <v>4132</v>
+        <v>1804</v>
       </c>
       <c r="E35" t="str">
-        <v>cartulina</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ModoDía 39</v>
+        <v>Kristel 21</v>
       </c>
       <c r="B36" t="str">
         <v>digital</v>
       </c>
       <c r="C36" t="str">
-        <v>A0</v>
+        <v>personalizado</v>
       </c>
       <c r="D36">
-        <v>343</v>
+        <v>119</v>
       </c>
       <c r="E36" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Smart Fit 44</v>
+        <v>Alejandro 27</v>
       </c>
       <c r="B37" t="str">
-        <v>gran_formato</v>
+        <v>offset</v>
       </c>
       <c r="C37" t="str">
-        <v>personalizado</v>
+        <v>A1</v>
       </c>
       <c r="D37">
-        <v>554</v>
+        <v>739</v>
       </c>
       <c r="E37" t="str">
-        <v>vinilo</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Tottus 56</v>
+        <v>Smart Fit 98</v>
       </c>
       <c r="B38" t="str">
-        <v>serigrafia</v>
+        <v>gran_formato</v>
       </c>
       <c r="C38" t="str">
-        <v>A0</v>
+        <v>A2</v>
       </c>
       <c r="D38">
-        <v>1668</v>
+        <v>977</v>
       </c>
       <c r="E38" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ModoDía 77</v>
+        <v>Jesus 46</v>
       </c>
       <c r="B39" t="str">
         <v>serigrafia</v>
       </c>
       <c r="C39" t="str">
-        <v>A2</v>
+        <v>personalizado</v>
       </c>
       <c r="D39">
-        <v>2511</v>
+        <v>1346</v>
       </c>
       <c r="E39" t="str">
-        <v>papel_couche</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Clínica Rene 25</v>
+        <v>ModoDía 44</v>
       </c>
       <c r="B40" t="str">
         <v>digital</v>
       </c>
       <c r="C40" t="str">
-        <v>A1</v>
+        <v>A4</v>
       </c>
       <c r="D40">
-        <v>876</v>
+        <v>4891</v>
       </c>
       <c r="E40" t="str">
-        <v>papel_couche</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Tottus 59</v>
+        <v>Jesus 37</v>
       </c>
       <c r="B41" t="str">
         <v>offset</v>
       </c>
       <c r="C41" t="str">
-        <v>A2</v>
+        <v>personalizado</v>
       </c>
       <c r="D41">
-        <v>1169</v>
+        <v>1431</v>
       </c>
       <c r="E41" t="str">
-        <v>papel_couche</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Alejandro 21</v>
+        <v>Noemi 99</v>
       </c>
       <c r="B42" t="str">
         <v>digital</v>
       </c>
       <c r="C42" t="str">
-        <v>personalizado</v>
+        <v>A0</v>
       </c>
       <c r="D42">
-        <v>4753</v>
+        <v>3973</v>
       </c>
       <c r="E42" t="str">
-        <v>lona</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Smart Fit 58</v>
+        <v>Jesus 15</v>
       </c>
       <c r="B43" t="str">
-        <v>serigrafia</v>
+        <v>gran_formato</v>
       </c>
       <c r="C43" t="str">
-        <v>personalizado</v>
+        <v>A0</v>
       </c>
       <c r="D43">
-        <v>4514</v>
+        <v>221</v>
       </c>
       <c r="E43" t="str">
-        <v>papel_couche</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Alejandro 27</v>
+        <v>Tottus 16</v>
       </c>
       <c r="B44" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C44" t="str">
-        <v>A3</v>
+        <v>A4</v>
       </c>
       <c r="D44">
-        <v>1138</v>
+        <v>2793</v>
       </c>
       <c r="E44" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Clínica Rene 32</v>
+        <v>Joselin 40</v>
       </c>
       <c r="B45" t="str">
-        <v>gran_formato</v>
+        <v>digital</v>
       </c>
       <c r="C45" t="str">
         <v>A0</v>
       </c>
       <c r="D45">
-        <v>2630</v>
+        <v>2253</v>
       </c>
       <c r="E45" t="str">
-        <v>papel_bond</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Joselin 73</v>
+        <v>UTP 86</v>
       </c>
       <c r="B46" t="str">
         <v>serigrafia</v>
       </c>
       <c r="C46" t="str">
-        <v>personalizado</v>
+        <v>A3</v>
       </c>
       <c r="D46">
-        <v>4406</v>
+        <v>3729</v>
       </c>
       <c r="E46" t="str">
-        <v>papel_couche</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Smart Fit 93</v>
+        <v>UTP 76</v>
       </c>
       <c r="B47" t="str">
-        <v>offset</v>
+        <v>digital</v>
       </c>
       <c r="C47" t="str">
-        <v>personalizado</v>
+        <v>A0</v>
       </c>
       <c r="D47">
-        <v>2587</v>
+        <v>2515</v>
       </c>
       <c r="E47" t="str">
-        <v>lona</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Joselin 59</v>
+        <v>Joselin 50</v>
       </c>
       <c r="B48" t="str">
-        <v>serigrafia</v>
+        <v>gran_formato</v>
       </c>
       <c r="C48" t="str">
-        <v>A2</v>
+        <v>personalizado</v>
       </c>
       <c r="D48">
-        <v>4234</v>
+        <v>1145</v>
       </c>
       <c r="E48" t="str">
-        <v>papel_couche</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Sofia 74</v>
+        <v>Kristel 4</v>
       </c>
       <c r="B49" t="str">
         <v>serigrafia</v>
       </c>
       <c r="C49" t="str">
-        <v>personalizado</v>
+        <v>A4</v>
       </c>
       <c r="D49">
-        <v>634</v>
+        <v>3055</v>
       </c>
       <c r="E49" t="str">
-        <v>lona</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Smart Fit 6</v>
+        <v>Tottus 93</v>
       </c>
       <c r="B50" t="str">
-        <v>serigrafia</v>
+        <v>digital</v>
       </c>
       <c r="C50" t="str">
-        <v>A4</v>
+        <v>A3</v>
       </c>
       <c r="D50">
-        <v>707</v>
+        <v>2045</v>
       </c>
       <c r="E50" t="str">
         <v>vinilo</v>
@@ -1251,16 +1251,16 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Clínica Rene 20</v>
+        <v>Jesus 36</v>
       </c>
       <c r="B51" t="str">
-        <v>gran_formato</v>
+        <v>digital</v>
       </c>
       <c r="C51" t="str">
-        <v>A0</v>
+        <v>A4</v>
       </c>
       <c r="D51">
-        <v>1583</v>
+        <v>4963</v>
       </c>
       <c r="E51" t="str">
         <v>papel_couche</v>
@@ -1268,67 +1268,67 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Kristel 43</v>
+        <v>Alejandro 77</v>
       </c>
       <c r="B52" t="str">
-        <v>offset</v>
+        <v>serigrafia</v>
       </c>
       <c r="C52" t="str">
-        <v>A4</v>
+        <v>A2</v>
       </c>
       <c r="D52">
-        <v>2394</v>
+        <v>2267</v>
       </c>
       <c r="E52" t="str">
-        <v>lona</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>UTP 24</v>
+        <v>UTP 88</v>
       </c>
       <c r="B53" t="str">
-        <v>gran_formato</v>
+        <v>serigrafia</v>
       </c>
       <c r="C53" t="str">
-        <v>A4</v>
+        <v>A2</v>
       </c>
       <c r="D53">
-        <v>721</v>
+        <v>2239</v>
       </c>
       <c r="E53" t="str">
-        <v>cartulina</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Joselin 26</v>
+        <v>Noemi 16</v>
       </c>
       <c r="B54" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C54" t="str">
-        <v>A2</v>
+        <v>A3</v>
       </c>
       <c r="D54">
-        <v>2536</v>
+        <v>1678</v>
       </c>
       <c r="E54" t="str">
-        <v>papel_bond</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Smart Fit 40</v>
+        <v>Alejandro 99</v>
       </c>
       <c r="B55" t="str">
-        <v>digital</v>
+        <v>gran_formato</v>
       </c>
       <c r="C55" t="str">
-        <v>A1</v>
+        <v>personalizado</v>
       </c>
       <c r="D55">
-        <v>3880</v>
+        <v>1315</v>
       </c>
       <c r="E55" t="str">
         <v>vinilo</v>
@@ -1336,135 +1336,135 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>UTP 10</v>
+        <v>Sofia 76</v>
       </c>
       <c r="B56" t="str">
-        <v>gran_formato</v>
+        <v>digital</v>
       </c>
       <c r="C56" t="str">
-        <v>personalizado</v>
+        <v>A4</v>
       </c>
       <c r="D56">
-        <v>4216</v>
+        <v>2502</v>
       </c>
       <c r="E56" t="str">
-        <v>cartulina</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Kristel 25</v>
+        <v>Clínica Rene 84</v>
       </c>
       <c r="B57" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C57" t="str">
         <v>A1</v>
       </c>
       <c r="D57">
-        <v>2312</v>
+        <v>3124</v>
       </c>
       <c r="E57" t="str">
-        <v>lona</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ModoDía 100</v>
+        <v>Smart Fit 46</v>
       </c>
       <c r="B58" t="str">
         <v>offset</v>
       </c>
       <c r="C58" t="str">
-        <v>A1</v>
+        <v>A2</v>
       </c>
       <c r="D58">
-        <v>2537</v>
+        <v>833</v>
       </c>
       <c r="E58" t="str">
-        <v>papel_couche</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Sofia 96</v>
+        <v>Alejandro 37</v>
       </c>
       <c r="B59" t="str">
-        <v>offset</v>
+        <v>serigrafia</v>
       </c>
       <c r="C59" t="str">
-        <v>A4</v>
+        <v>A3</v>
       </c>
       <c r="D59">
-        <v>4040</v>
+        <v>809</v>
       </c>
       <c r="E59" t="str">
-        <v>vinilo</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Smart Fit 61</v>
+        <v>Alejandro 80</v>
       </c>
       <c r="B60" t="str">
-        <v>digital</v>
+        <v>serigrafia</v>
       </c>
       <c r="C60" t="str">
-        <v>A3</v>
+        <v>personalizado</v>
       </c>
       <c r="D60">
-        <v>296</v>
+        <v>4651</v>
       </c>
       <c r="E60" t="str">
-        <v>vinilo</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Sofia 26</v>
+        <v>Alejandro 63</v>
       </c>
       <c r="B61" t="str">
-        <v>gran_formato</v>
+        <v>serigrafia</v>
       </c>
       <c r="C61" t="str">
         <v>A2</v>
       </c>
       <c r="D61">
-        <v>1978</v>
+        <v>361</v>
       </c>
       <c r="E61" t="str">
-        <v>cartulina</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ModoDía 45</v>
+        <v>Sofia 52</v>
       </c>
       <c r="B62" t="str">
-        <v>gran_formato</v>
+        <v>serigrafia</v>
       </c>
       <c r="C62" t="str">
         <v>A4</v>
       </c>
       <c r="D62">
-        <v>2997</v>
+        <v>1262</v>
       </c>
       <c r="E62" t="str">
-        <v>lona</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>UTP 63</v>
+        <v>Joselin 86</v>
       </c>
       <c r="B63" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C63" t="str">
-        <v>A1</v>
+        <v>A0</v>
       </c>
       <c r="D63">
-        <v>2619</v>
+        <v>115</v>
       </c>
       <c r="E63" t="str">
         <v>lona</v>
@@ -1472,101 +1472,101 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Kristel 95</v>
+        <v>Noemi 63</v>
       </c>
       <c r="B64" t="str">
-        <v>digital</v>
+        <v>gran_formato</v>
       </c>
       <c r="C64" t="str">
-        <v>personalizado</v>
+        <v>A0</v>
       </c>
       <c r="D64">
-        <v>2249</v>
+        <v>894</v>
       </c>
       <c r="E64" t="str">
-        <v>papel_couche</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Kristel 83</v>
+        <v>Alejandro 77</v>
       </c>
       <c r="B65" t="str">
         <v>digital</v>
       </c>
       <c r="C65" t="str">
-        <v>A1</v>
+        <v>A3</v>
       </c>
       <c r="D65">
-        <v>3471</v>
+        <v>830</v>
       </c>
       <c r="E65" t="str">
-        <v>vinilo</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Joselin 100</v>
+        <v>Noemi 7</v>
       </c>
       <c r="B66" t="str">
-        <v>digital</v>
+        <v>gran_formato</v>
       </c>
       <c r="C66" t="str">
-        <v>A1</v>
+        <v>personalizado</v>
       </c>
       <c r="D66">
-        <v>4078</v>
+        <v>740</v>
       </c>
       <c r="E66" t="str">
-        <v>lona</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Sofia 35</v>
+        <v>Noemi 64</v>
       </c>
       <c r="B67" t="str">
         <v>digital</v>
       </c>
       <c r="C67" t="str">
-        <v>personalizado</v>
+        <v>A4</v>
       </c>
       <c r="D67">
-        <v>4269</v>
+        <v>3481</v>
       </c>
       <c r="E67" t="str">
-        <v>papel_bond</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Smart Fit 4</v>
+        <v>Noemi 14</v>
       </c>
       <c r="B68" t="str">
-        <v>offset</v>
+        <v>gran_formato</v>
       </c>
       <c r="C68" t="str">
-        <v>A1</v>
+        <v>A0</v>
       </c>
       <c r="D68">
-        <v>1477</v>
+        <v>4379</v>
       </c>
       <c r="E68" t="str">
-        <v>cartulina</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Tottus 43</v>
+        <v>Smart Fit 75</v>
       </c>
       <c r="B69" t="str">
         <v>gran_formato</v>
       </c>
       <c r="C69" t="str">
-        <v>A0</v>
+        <v>A4</v>
       </c>
       <c r="D69">
-        <v>878</v>
+        <v>1455</v>
       </c>
       <c r="E69" t="str">
         <v>papel_bond</v>
@@ -1574,7 +1574,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Joselin 15</v>
+        <v>Alejandro 86</v>
       </c>
       <c r="B70" t="str">
         <v>offset</v>
@@ -1583,49 +1583,49 @@
         <v>A2</v>
       </c>
       <c r="D70">
-        <v>4110</v>
+        <v>1255</v>
       </c>
       <c r="E70" t="str">
-        <v>cartulina</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Noemi 83</v>
+        <v>Jesus 9</v>
       </c>
       <c r="B71" t="str">
-        <v>offset</v>
+        <v>digital</v>
       </c>
       <c r="C71" t="str">
         <v>A0</v>
       </c>
       <c r="D71">
-        <v>1018</v>
+        <v>3886</v>
       </c>
       <c r="E71" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>UTP 5</v>
+        <v>Alejandro 21</v>
       </c>
       <c r="B72" t="str">
-        <v>offset</v>
+        <v>digital</v>
       </c>
       <c r="C72" t="str">
-        <v>A0</v>
+        <v>personalizado</v>
       </c>
       <c r="D72">
-        <v>2349</v>
+        <v>3692</v>
       </c>
       <c r="E72" t="str">
-        <v>cartulina</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Alejandro 49</v>
+        <v>ModoDía 99</v>
       </c>
       <c r="B73" t="str">
         <v>gran_formato</v>
@@ -1634,15 +1634,15 @@
         <v>A1</v>
       </c>
       <c r="D73">
-        <v>4706</v>
+        <v>118</v>
       </c>
       <c r="E73" t="str">
-        <v>papel_bond</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Tottus 66</v>
+        <v>Sofia 82</v>
       </c>
       <c r="B74" t="str">
         <v>gran_formato</v>
@@ -1651,24 +1651,24 @@
         <v>A3</v>
       </c>
       <c r="D74">
-        <v>4280</v>
+        <v>4757</v>
       </c>
       <c r="E74" t="str">
-        <v>cartulina</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>UTP 54</v>
+        <v>Sofia 67</v>
       </c>
       <c r="B75" t="str">
-        <v>gran_formato</v>
+        <v>serigrafia</v>
       </c>
       <c r="C75" t="str">
-        <v>A0</v>
+        <v>A3</v>
       </c>
       <c r="D75">
-        <v>3840</v>
+        <v>4112</v>
       </c>
       <c r="E75" t="str">
         <v>papel_bond</v>
@@ -1676,16 +1676,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Tottus 30</v>
+        <v>Smart Fit 76</v>
       </c>
       <c r="B76" t="str">
         <v>digital</v>
       </c>
       <c r="C76" t="str">
-        <v>A2</v>
+        <v>A4</v>
       </c>
       <c r="D76">
-        <v>2256</v>
+        <v>3677</v>
       </c>
       <c r="E76" t="str">
         <v>papel_bond</v>
@@ -1693,33 +1693,33 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Kristel 83</v>
+        <v>Kristel 55</v>
       </c>
       <c r="B77" t="str">
-        <v>gran_formato</v>
+        <v>offset</v>
       </c>
       <c r="C77" t="str">
         <v>A2</v>
       </c>
       <c r="D77">
-        <v>1809</v>
+        <v>4220</v>
       </c>
       <c r="E77" t="str">
-        <v>cartulina</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Sofia 36</v>
+        <v>Clínica Rene 65</v>
       </c>
       <c r="B78" t="str">
-        <v>offset</v>
+        <v>serigrafia</v>
       </c>
       <c r="C78" t="str">
-        <v>A4</v>
+        <v>A1</v>
       </c>
       <c r="D78">
-        <v>4621</v>
+        <v>2057</v>
       </c>
       <c r="E78" t="str">
         <v>vinilo</v>
@@ -1727,101 +1727,101 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Smart Fit 61</v>
+        <v>Kristel 61</v>
       </c>
       <c r="B79" t="str">
-        <v>serigrafia</v>
+        <v>gran_formato</v>
       </c>
       <c r="C79" t="str">
-        <v>A1</v>
+        <v>personalizado</v>
       </c>
       <c r="D79">
-        <v>4188</v>
+        <v>47</v>
       </c>
       <c r="E79" t="str">
-        <v>papel_couche</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Alejandro 92</v>
+        <v>Kristel 36</v>
       </c>
       <c r="B80" t="str">
-        <v>offset</v>
+        <v>digital</v>
       </c>
       <c r="C80" t="str">
-        <v>A2</v>
+        <v>A3</v>
       </c>
       <c r="D80">
-        <v>3317</v>
+        <v>3540</v>
       </c>
       <c r="E80" t="str">
-        <v>papel_couche</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Joselin 18</v>
+        <v>Tottus 14</v>
       </c>
       <c r="B81" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C81" t="str">
-        <v>A3</v>
+        <v>A1</v>
       </c>
       <c r="D81">
-        <v>28</v>
+        <v>1063</v>
       </c>
       <c r="E81" t="str">
-        <v>cartulina</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Jesus 100</v>
+        <v>Tottus 59</v>
       </c>
       <c r="B82" t="str">
-        <v>serigrafia</v>
+        <v>gran_formato</v>
       </c>
       <c r="C82" t="str">
-        <v>A2</v>
+        <v>personalizado</v>
       </c>
       <c r="D82">
-        <v>1766</v>
+        <v>2765</v>
       </c>
       <c r="E82" t="str">
-        <v>lona</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Smart Fit 78</v>
+        <v>Smart Fit 29</v>
       </c>
       <c r="B83" t="str">
-        <v>offset</v>
+        <v>gran_formato</v>
       </c>
       <c r="C83" t="str">
-        <v>A0</v>
+        <v>A2</v>
       </c>
       <c r="D83">
-        <v>2077</v>
+        <v>4874</v>
       </c>
       <c r="E83" t="str">
-        <v>vinilo</v>
+        <v>lona</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Tottus 47</v>
+        <v>Smart Fit 81</v>
       </c>
       <c r="B84" t="str">
         <v>digital</v>
       </c>
       <c r="C84" t="str">
-        <v>A1</v>
+        <v>A0</v>
       </c>
       <c r="D84">
-        <v>2297</v>
+        <v>2327</v>
       </c>
       <c r="E84" t="str">
         <v>papel_couche</v>
@@ -1829,109 +1829,109 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Jesus 79</v>
+        <v>Sofia 78</v>
       </c>
       <c r="B85" t="str">
-        <v>offset</v>
+        <v>digital</v>
       </c>
       <c r="C85" t="str">
-        <v>personalizado</v>
+        <v>A1</v>
       </c>
       <c r="D85">
-        <v>1589</v>
+        <v>4446</v>
       </c>
       <c r="E85" t="str">
-        <v>papel_couche</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Jesus 2</v>
+        <v>ModoDía 23</v>
       </c>
       <c r="B86" t="str">
-        <v>gran_formato</v>
+        <v>serigrafia</v>
       </c>
       <c r="C86" t="str">
-        <v>A3</v>
+        <v>A2</v>
       </c>
       <c r="D86">
-        <v>816</v>
+        <v>660</v>
       </c>
       <c r="E86" t="str">
-        <v>lona</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Tottus 81</v>
+        <v>UTP 19</v>
       </c>
       <c r="B87" t="str">
         <v>digital</v>
       </c>
       <c r="C87" t="str">
-        <v>A4</v>
+        <v>personalizado</v>
       </c>
       <c r="D87">
-        <v>1619</v>
+        <v>4168</v>
       </c>
       <c r="E87" t="str">
-        <v>cartulina</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Alejandro 17</v>
+        <v>Sofia 7</v>
       </c>
       <c r="B88" t="str">
-        <v>gran_formato</v>
+        <v>digital</v>
       </c>
       <c r="C88" t="str">
-        <v>A4</v>
+        <v>A2</v>
       </c>
       <c r="D88">
-        <v>881</v>
+        <v>2906</v>
       </c>
       <c r="E88" t="str">
-        <v>vinilo</v>
+        <v>papel_couche</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Tottus 2</v>
+        <v>Jesus 86</v>
       </c>
       <c r="B89" t="str">
-        <v>digital</v>
+        <v>offset</v>
       </c>
       <c r="C89" t="str">
-        <v>A3</v>
+        <v>A2</v>
       </c>
       <c r="D89">
-        <v>3287</v>
+        <v>1364</v>
       </c>
       <c r="E89" t="str">
-        <v>papel_couche</v>
+        <v>papel_bond</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Kristel 91</v>
+        <v>Kristel 53</v>
       </c>
       <c r="B90" t="str">
-        <v>serigrafia</v>
+        <v>offset</v>
       </c>
       <c r="C90" t="str">
-        <v>A0</v>
+        <v>A1</v>
       </c>
       <c r="D90">
-        <v>4119</v>
+        <v>3288</v>
       </c>
       <c r="E90" t="str">
-        <v>papel_bond</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Alejandro 81</v>
+        <v>ModoDía 67</v>
       </c>
       <c r="B91" t="str">
         <v>digital</v>
@@ -1940,58 +1940,58 @@
         <v>A2</v>
       </c>
       <c r="D91">
-        <v>3237</v>
+        <v>4788</v>
       </c>
       <c r="E91" t="str">
-        <v>lona</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Sofia 4</v>
+        <v>Kristel 91</v>
       </c>
       <c r="B92" t="str">
         <v>digital</v>
       </c>
       <c r="C92" t="str">
-        <v>A1</v>
+        <v>personalizado</v>
       </c>
       <c r="D92">
-        <v>4282</v>
+        <v>3589</v>
       </c>
       <c r="E92" t="str">
-        <v>papel_couche</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Tottus 78</v>
+        <v>Alejandro 76</v>
       </c>
       <c r="B93" t="str">
-        <v>offset</v>
+        <v>digital</v>
       </c>
       <c r="C93" t="str">
-        <v>A1</v>
+        <v>A4</v>
       </c>
       <c r="D93">
-        <v>1715</v>
+        <v>3394</v>
       </c>
       <c r="E93" t="str">
-        <v>papel_bond</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Joselin 3</v>
+        <v>Sofia 48</v>
       </c>
       <c r="B94" t="str">
-        <v>gran_formato</v>
+        <v>offset</v>
       </c>
       <c r="C94" t="str">
-        <v>A0</v>
+        <v>A1</v>
       </c>
       <c r="D94">
-        <v>1562</v>
+        <v>4407</v>
       </c>
       <c r="E94" t="str">
         <v>cartulina</v>
@@ -1999,16 +1999,16 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Tottus 64</v>
+        <v>ModoDía 68</v>
       </c>
       <c r="B95" t="str">
         <v>gran_formato</v>
       </c>
       <c r="C95" t="str">
-        <v>A3</v>
+        <v>A0</v>
       </c>
       <c r="D95">
-        <v>1704</v>
+        <v>1816</v>
       </c>
       <c r="E95" t="str">
         <v>lona</v>
@@ -2016,84 +2016,84 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Noemi 65</v>
+        <v>UTP 72</v>
       </c>
       <c r="B96" t="str">
-        <v>gran_formato</v>
+        <v>digital</v>
       </c>
       <c r="C96" t="str">
-        <v>A1</v>
+        <v>A0</v>
       </c>
       <c r="D96">
-        <v>4672</v>
+        <v>308</v>
       </c>
       <c r="E96" t="str">
-        <v>papel_bond</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Jesus 11</v>
+        <v>Kristel 3</v>
       </c>
       <c r="B97" t="str">
-        <v>serigrafia</v>
+        <v>gran_formato</v>
       </c>
       <c r="C97" t="str">
-        <v>A3</v>
+        <v>A1</v>
       </c>
       <c r="D97">
-        <v>2262</v>
+        <v>1931</v>
       </c>
       <c r="E97" t="str">
-        <v>papel_couche</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Noemi 5</v>
+        <v>Noemi 34</v>
       </c>
       <c r="B98" t="str">
-        <v>gran_formato</v>
+        <v>serigrafia</v>
       </c>
       <c r="C98" t="str">
-        <v>A4</v>
+        <v>personalizado</v>
       </c>
       <c r="D98">
-        <v>2707</v>
+        <v>2862</v>
       </c>
       <c r="E98" t="str">
-        <v>lona</v>
+        <v>cartulina</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Sofia 57</v>
+        <v>Jesus 26</v>
       </c>
       <c r="B99" t="str">
-        <v>digital</v>
+        <v>gran_formato</v>
       </c>
       <c r="C99" t="str">
-        <v>A3</v>
+        <v>A1</v>
       </c>
       <c r="D99">
-        <v>3261</v>
+        <v>1562</v>
       </c>
       <c r="E99" t="str">
-        <v>papel_bond</v>
+        <v>vinilo</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Smart Fit 77</v>
+        <v>Joselin 43</v>
       </c>
       <c r="B100" t="str">
         <v>digital</v>
       </c>
       <c r="C100" t="str">
-        <v>A2</v>
+        <v>personalizado</v>
       </c>
       <c r="D100">
-        <v>1051</v>
+        <v>3969</v>
       </c>
       <c r="E100" t="str">
         <v>vinilo</v>
@@ -2101,19 +2101,19 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Joselin 56</v>
+        <v>Kristel 14</v>
       </c>
       <c r="B101" t="str">
-        <v>digital</v>
+        <v>gran_formato</v>
       </c>
       <c r="C101" t="str">
-        <v>A2</v>
+        <v>A3</v>
       </c>
       <c r="D101">
-        <v>1400</v>
+        <v>2144</v>
       </c>
       <c r="E101" t="str">
-        <v>papel_couche</v>
+        <v>lona</v>
       </c>
     </row>
   </sheetData>

</xml_diff>